<commit_message>
Update Data Quality Issue Log
</commit_message>
<xml_diff>
--- a/Enova_Issue_Log.xlsx
+++ b/Enova_Issue_Log.xlsx
@@ -8,16 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://postidcac-my.sharepoint.com/personal/roei_tsahi_post_runi_ac_il/Documents/Desktop/1 PROJECT/אני/דאטא סופי/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="11_F25DC773A252ABDACC1048FBE95E48A25BDE58E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{498ED05A-AA89-4B58-9D77-9AF3D3E626F0}"/>
+  <xr:revisionPtr revIDLastSave="95" documentId="11_F25DC773A252ABDACC1048FBE95E48A25BDE58E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D27AB8FB-F906-48F5-94E9-E9BDA02B0EBB}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -210,34 +207,33 @@
     <t>ORDER_ID</t>
   </si>
   <si>
-    <t>Significant Row-Level Redundancy &amp; Broken Granularity: Identified 15,196 exact duplicates (14.05% of dataset) where every column value was identical. The current Order-Product granularity creates severe ambiguity: without a LINE_ITEM_ID or QUANTITY column, it is mathematically impossible to distinguish a technical "double-firing" logging bug from a legitimate purchase of multiple identical items. This poses a major risk for revenue overestimation and analytical bias.</t>
-  </si>
-  <si>
-    <t>1. Business Decision: A 14% exact-duplicate rate is statistically improbable and strongly indicates a system error. I opted to deduplicate these records to prevent severe revenue inflation and protect KPI integrity.
-2. Action Taken (SQL Logic): Because standard keys were useless, I executed a surgical deduplication using a SQL CTE with the ROW_NUMBER() window function, partitioned by all columns. Filtering to retain only the first instance (rn = 1) safely collapsed identical retries while retaining unique records.
-3. Escalation: In a production environment, before any massive data removal, I would cross-reference these anomalous ORDER_IDs with the payment gateway (e.g., Stripe) to verify actual captured funds. I would then escalate to Data Engineering to investigate the root cause and implement API idempotency keys.</t>
-  </si>
-  <si>
     <t>LOYALTY_PROGRAM</t>
   </si>
   <si>
-    <t>SCD (Slowly Changing Dimension) Ambiguity: 1,026 Users appear with mixed statuses (both '0' and '1') across different orders. This prevents static classification of users as strictly "Member" or "Non-Member" for their entire lifetime.</t>
-  </si>
-  <si>
-    <t>Adopted a Dual-Attribution approach to bypass SCD Limitations:  Due to the absence of a continuous history table (SCD Type 2 for loyalty_program with 'Valid_From' and 'Valid_To' timestamps), I mitigated this without distorting the data by applying two rules:
-1. Transaction-Based: Instead of static user classification (which introduces Look-Ahead Bias), financial metrics (Revenue/AOV) are attributed to the exact loyalty status at the moment of purchase.
-2. Ever-Member (Cohort): Utilized exclusively for behavioral metrics (Stickiness) to track long-term cadence, regardless of point-in-time toggling.
-Strategic Flag to Data Engineering: Recommended implementing an SCD Type 2 tracking table for the loyalty_program field. Logging the exact start and end dates of a user's loyalty status will enable precise, continuous state tracking for future retention and churn modeling.</t>
-  </si>
-  <si>
     <t>CREATED_ON</t>
   </si>
   <si>
-    <t>Data Integrity Violation (Immutable Field Update): Logic dictates 'Account Creation' should be a one-time, immutable event. Analysis revealed 4,816 users with multiple conflicting creation dates, suggesting the field is being overwritten and lacks logical consistency.</t>
-  </si>
-  <si>
-    <t>Excluded from Time-Based Analysis: Retained original values but deemed the field unreliable for 'Time-to-Conversion' or 'Customer Lifetime' metrics. Scrapping these analyses prevented Look-Ahead Bias and misleading Cohort Retention results.
-Data Sleuthing &amp; Escalation: SQL tests confirmed this is an independent system bug by isolating users whose Loyalty Status remained completely static, yet their CREATED_ON dates still fluctuated and even regressed chronologically. Flagged to IT/Engineering to implement a permanent, append-only Created_At timestamp.</t>
+    <t>Potential Row-Level Duplication &amp; Unresolved Grain: Identified 15,196 exact duplicate-like records (14.05% of the dataset), where all available fields were identical. Because the source lacks both a LINE_ITEM_ID and QUANTITY field, the available grain cannot reliably distinguish duplicated source events from legitimate purchases of multiple identical items. Removing these records without external validation could therefore understate revenue and item volume.</t>
+  </si>
+  <si>
+    <t>1. Analytical Decision: Retained all duplicate-like records because the available source grain was insufficient to validate them as true duplicates.
+2. SQL Diagnostic: Used a ROW_NUMBER() window function across all available fields to isolate exact duplicate candidates for investigation. The diagnostic was not used to remove records from the analytical dataset.
+3. Production Follow-up: Validate candidate records against the order-management and payment source before deletion. If a reliable LINE_ITEM_ID is available, ORDER_ID + LINE_ITEM_ID should serve as the primary duplicate-validation key, with ROW_NUMBER() used to identify repeated keys. Data Engineering should also enforce the intended source grain and appropriate uniqueness/idempotency controls upstream.</t>
+  </si>
+  <si>
+    <t>Loyalty Status History Ambiguity (SCD Limitation): 1,026 users appear with both 0 and 1 loyalty values across different transactions. Without an effective-dated membership history, users cannot be reliably classified under a single lifetime status or their exact membership state reconstructed across the full historical timeline.</t>
+  </si>
+  <si>
+    <t>1. Analytical Treatment: Used the loyalty value recorded on each transaction for transaction-level financial reporting such as Revenue and AOV. For long-term behavioral comparisons, a separately defined retrospective Ever-Member cohort was used. The two analytical views were kept separate and were not presented as a reconstructed historical membership timeline.
+2. Production Follow-up: Data Engineering should maintain an effective-dated loyalty history, such as an SCD Type 2 or membership-event table containing Valid_From and Valid_To fields. This would support reliable historical membership attribution and future retention/churn analysis.</t>
+  </si>
+  <si>
+    <t>Account Creation Date Integrity Violation: Analysis identified 4,816 users with multiple conflicting CREATED_ON values, including cases where dates regressed chronologically. Because account creation should represent a single immutable event, the field cannot be treated as a reliable account-start timestamp.</t>
+  </si>
+  <si>
+    <t>1. Analytical Decision: Retained the affected records because removing complete transactions due to an unreliable CREATED_ON field would unnecessarily bias otherwise valid sales and order analysis.
+2. Analytical Limitation: The unreliable account-creation timestamp prevented reliable tenure-based analysis, including time-to-conversion, Lifetime Value (LTV), and cohort retention.
+3. Validation &amp; Production Follow-up: SQL checks showed that CREATED_ON inconsistencies persisted even among users whose loyalty status remained unchanged, confirming that the issue was not explained by loyalty-status changes. In a production environment, the source-system owner / Data Engineering team should validate and persist a canonical, immutable ACCOUNT_CREATED_AT timestamp for downstream analytics.</t>
   </si>
 </sst>
 </file>
@@ -246,8 +242,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="168" formatCode="0.000%"/>
-    <numFmt numFmtId="169" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="0.000%"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -306,7 +302,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -315,29 +311,40 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -346,15 +353,6 @@
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="15">
-    <dxf>
-      <alignment vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -372,20 +370,83 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="168" formatCode="0.000%"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="164" formatCode="0.000%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -412,60 +473,6 @@
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -479,40 +486,22 @@
 </styleSheet>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Orders_Raw"/>
-      <sheetName val="Country_Region_Lookup_raw"/>
-      <sheetName val="Issue Log"/>
-      <sheetName val="Country_Region_Cleaned"/>
-      <sheetName val="Orders_Final_Cleaned"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{435BDB28-E81B-4B25-BDD0-C7DCCF9788EA}" name="Table7" displayName="Table7" ref="A1:G19" totalsRowShown="0" headerRowDxfId="8" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{435BDB28-E81B-4B25-BDD0-C7DCCF9788EA}" name="Table7" displayName="Table7" ref="A1:G19" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{CFD2519F-D72A-4C93-9575-12533EB1B1B9}" name="table" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{EFABAC00-2EDD-44E7-9550-9F1F735C3D69}" name="column" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{1699682E-5B59-4C23-B936-92FE3B2BA111}" name="issue" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{4B28B51F-7AB2-4917-ABEF-36A2CA9B9841}" name="row count" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{D2576707-0D31-430A-AC19-364C209108A7}" name="magnitude" dataDxfId="3" dataCellStyle="Percent"/>
-    <tableColumn id="6" xr3:uid="{61AAC634-A46B-41B3-8E90-12E92A2F1404}" name="solvable?" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{3B04A96D-4145-4AE1-A3D4-E2CBAA67D204}" name="resolution" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{CFD2519F-D72A-4C93-9575-12533EB1B1B9}" name="table" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{EFABAC00-2EDD-44E7-9550-9F1F735C3D69}" name="column" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{1699682E-5B59-4C23-B936-92FE3B2BA111}" name="issue" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{4B28B51F-7AB2-4917-ABEF-36A2CA9B9841}" name="row count" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{D2576707-0D31-430A-AC19-364C209108A7}" name="magnitude" dataDxfId="0" dataCellStyle="Percent">
+      <calculatedColumnFormula>Table7[[#This Row],[row count]]/108127</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{61AAC634-A46B-41B3-8E90-12E92A2F1404}" name="solvable?" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{3B04A96D-4145-4AE1-A3D4-E2CBAA67D204}" name="resolution" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -823,20 +812,20 @@
       <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="9">
         <v>27</v>
       </c>
-      <c r="E2" s="7">
-        <f>D2/COUNTA([1]!Table13[USER_ID])</f>
+      <c r="E2" s="10">
+        <f>Table7[[#This Row],[row count]]/108127</f>
         <v>2.4970636381292367E-4</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="4" t="s">
         <v>11</v>
       </c>
     </row>
@@ -847,20 +836,20 @@
       <c r="B3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="9">
         <v>3</v>
       </c>
-      <c r="E3" s="7">
-        <f>D3/COUNTA([1]!Table13[USER_ID])</f>
+      <c r="E3" s="10">
+        <f>Table7[[#This Row],[row count]]/108127</f>
         <v>2.77451515347693E-5</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="7" t="s">
         <v>14</v>
       </c>
     </row>
@@ -868,22 +857,22 @@
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="5" t="s">
         <v>18</v>
       </c>
     </row>
@@ -894,20 +883,20 @@
       <c r="B5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="9">
         <v>27</v>
       </c>
-      <c r="E5" s="7">
-        <f>D5/COUNTA([1]!Table13[USER_ID])</f>
+      <c r="E5" s="10">
+        <f>Table7[[#This Row],[row count]]/108127</f>
         <v>2.4970636381292367E-4</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="7" t="s">
         <v>21</v>
       </c>
     </row>
@@ -918,20 +907,20 @@
       <c r="B6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="9">
         <v>5379</v>
       </c>
-      <c r="E6" s="7">
-        <f>D6/COUNTA([1]!Table13[USER_ID])</f>
+      <c r="E6" s="10">
+        <f>Table7[[#This Row],[row count]]/108127</f>
         <v>4.9747056701841354E-2</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="5" t="s">
         <v>24</v>
       </c>
     </row>
@@ -942,16 +931,16 @@
       <c r="B7" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="9" t="s">
         <v>10</v>
       </c>
       <c r="G7" s="8" t="s">
@@ -965,20 +954,20 @@
       <c r="B8" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="9">
         <v>23435</v>
       </c>
-      <c r="E8" s="7">
-        <f>D8/COUNTA([1]!Table13[USER_ID])</f>
+      <c r="E8" s="10">
+        <f>Table7[[#This Row],[row count]]/108127</f>
         <v>0.21673587540577285</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="7" t="s">
         <v>30</v>
       </c>
     </row>
@@ -989,20 +978,20 @@
       <c r="B9" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="9">
         <v>158</v>
       </c>
-      <c r="E9" s="7">
-        <f>D9/COUNTA([1]!Table13[USER_ID])</f>
+      <c r="E9" s="10">
+        <f>Table7[[#This Row],[row count]]/108127</f>
         <v>1.4612446474978498E-3</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="7" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1013,20 +1002,20 @@
       <c r="B10" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="9">
         <v>1387</v>
       </c>
-      <c r="E10" s="7">
-        <f>D10/COUNTA([1]!Table13[USER_ID])</f>
+      <c r="E10" s="10">
+        <f>Table7[[#This Row],[row count]]/108127</f>
         <v>1.2827508392908339E-2</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F10" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="G10" s="5" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1037,20 +1026,20 @@
       <c r="B11" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="9">
         <v>1469</v>
       </c>
-      <c r="E11" s="7">
-        <f>D11/COUNTA([1]!Table13[USER_ID])</f>
+      <c r="E11" s="10">
+        <f>Table7[[#This Row],[row count]]/108127</f>
         <v>1.3585875868192033E-2</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G11" s="5" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1061,20 +1050,20 @@
       <c r="B12" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="9">
         <v>1387</v>
       </c>
-      <c r="E12" s="7">
-        <f>D12/COUNTA([1]!Table13[USER_ID])</f>
+      <c r="E12" s="10">
+        <f>Table7[[#This Row],[row count]]/108127</f>
         <v>1.2827508392908339E-2</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="G12" s="5" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1085,20 +1074,20 @@
       <c r="B13" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="9">
         <v>4287</v>
       </c>
-      <c r="E13" s="7">
-        <f>D13/COUNTA([1]!Table13[USER_ID])</f>
+      <c r="E13" s="10">
+        <f>Table7[[#This Row],[row count]]/108127</f>
         <v>3.964782154318533E-2</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="F13" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="G13" s="5" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1109,20 +1098,20 @@
       <c r="B14" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="9">
         <v>162</v>
       </c>
-      <c r="E14" s="7">
-        <f>D14/COUNTA([1]!Table13[USER_ID])</f>
+      <c r="E14" s="10">
+        <f>Table7[[#This Row],[row count]]/108127</f>
         <v>1.4982381828775421E-3</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="F14" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="G14" s="5" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1133,20 +1122,20 @@
       <c r="B15" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="9">
         <v>2</v>
       </c>
-      <c r="E15" s="7">
-        <f>D15/COUNTA([1]!Table13[USER_ID])</f>
+      <c r="E15" s="10">
+        <f>Table7[[#This Row],[row count]]/108127</f>
         <v>1.8496767689846199E-5</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="F15" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="G15" s="7" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1157,121 +1146,124 @@
       <c r="B16" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="9">
         <v>1</v>
       </c>
-      <c r="E16" s="7">
-        <f>D16/COUNTA([1]!Table13[USER_ID])</f>
+      <c r="E16" s="10">
+        <f>Table7[[#This Row],[row count]]/108127</f>
         <v>9.2483838449230996E-6</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="F16" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="7" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="187.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D17" s="11">
+        <v>15196</v>
+      </c>
+      <c r="E17" s="10">
+        <f>Table7[[#This Row],[row count]]/108127</f>
+        <v>0.14053844090745143</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="144" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D17" s="9">
-        <v>15196</v>
-      </c>
-      <c r="E17" s="7">
-        <f>D17/COUNTA([1]!Table13[USER_ID])</f>
-        <v>0.14053844090745143</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="G17" s="5" t="s">
+      <c r="C18" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D18" s="12">
+        <v>1026</v>
+      </c>
+      <c r="E18" s="10">
+        <f>Table7[[#This Row],[row count]]/108127</f>
+        <v>9.4888418248910995E-3</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D18" s="10">
-        <v>1026</v>
-      </c>
-      <c r="E18" s="7">
-        <f>D18/COUNTA([1]!Table13[USER_ID])</f>
-        <v>9.4888418248910995E-3</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="12">
         <v>4816</v>
       </c>
-      <c r="E19" s="11">
-        <f>D19/COUNTA([1]!Table13[USER_ID])</f>
+      <c r="E19" s="13">
+        <f>Table7[[#This Row],[row count]]/108127</f>
         <v>4.454021659714965E-2</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="F19" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G19" s="3" t="s">
+      <c r="G19" s="5" t="s">
         <v>63</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A18:A19 E18:E19">
-    <cfRule type="expression" dxfId="14" priority="3">
+    <cfRule type="expression" dxfId="8" priority="3">
       <formula>$F18="NO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="4">
+    <cfRule type="expression" dxfId="7" priority="4">
       <formula>$F18="YES"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:G19">
-    <cfRule type="expression" dxfId="12" priority="5">
+    <cfRule type="expression" dxfId="6" priority="5">
       <formula>$F2="NO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="6">
+    <cfRule type="expression" dxfId="5" priority="6">
       <formula>$F2="YES"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F18">
-    <cfRule type="expression" dxfId="10" priority="1">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>$F18="NO"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>$F18="YES"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="E4 E7" calculatedColumn="1"/>
+  </ignoredErrors>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>